<commit_message>
recalculate initial results against human3
</commit_message>
<xml_diff>
--- a/src/results/human/human_results_for_presentation.xlsx
+++ b/src/results/human/human_results_for_presentation.xlsx
@@ -8,25 +8,37 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\repos\Using-LLM-for-automated-feedback-generation-on-a-bachelor-thesis\src\results\human\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDD66748-D211-4FB1-B775-A94067A948E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{965EED26-06FB-4A40-B5F1-4B958FD99802}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="15" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Original" sheetId="1" r:id="rId1"/>
     <sheet name="Transformed" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet1" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="33">
   <si>
     <t>Question</t>
   </si>
@@ -125,9 +137,6 @@
   </si>
   <si>
     <t>Language</t>
-  </si>
-  <si>
-    <t>?</t>
   </si>
 </sst>
 </file>
@@ -808,7 +817,6 @@
           </c:extLst>
         </c:ser>
         <c:dLbls>
-          <c:dLblPos val="outEnd"/>
           <c:showLegendKey val="0"/>
           <c:showVal val="0"/>
           <c:showCatName val="0"/>
@@ -3439,7 +3447,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C9FC88B4-BAD5-4224-8F8B-E42023CF87E4}">
-  <dimension ref="A1:Y48"/>
+  <dimension ref="A1:Y45"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.7109375" style="3" customWidth="1"/>
@@ -4811,12 +4819,6 @@
       <c r="G30" s="5">
         <v>0.75433650914135697</v>
       </c>
-      <c r="K30" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="L30" s="3" t="s">
-        <v>31</v>
-      </c>
       <c r="O30"/>
     </row>
     <row r="31" spans="1:25" x14ac:dyDescent="0.25">
@@ -4841,12 +4843,6 @@
       <c r="G31" s="5">
         <v>0.69410473022319796</v>
       </c>
-      <c r="K31" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="L31" s="3" t="s">
-        <v>31</v>
-      </c>
       <c r="O31"/>
     </row>
     <row r="32" spans="1:25" x14ac:dyDescent="0.25">
@@ -4871,12 +4867,6 @@
       <c r="G32" s="5">
         <v>0.59314412363964997</v>
       </c>
-      <c r="K32" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="L32" s="3" t="s">
-        <v>31</v>
-      </c>
       <c r="O32"/>
     </row>
     <row r="33" spans="1:15" x14ac:dyDescent="0.25">
@@ -4901,12 +4891,6 @@
       <c r="G33" s="5">
         <v>0.29080080483815601</v>
       </c>
-      <c r="K33" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="L33" s="3" t="s">
-        <v>31</v>
-      </c>
       <c r="O33"/>
     </row>
     <row r="34" spans="1:15" x14ac:dyDescent="0.25">
@@ -4931,12 +4915,6 @@
       <c r="G34" s="5">
         <v>0.40883815970729898</v>
       </c>
-      <c r="K34" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="L34" s="3" t="s">
-        <v>31</v>
-      </c>
     </row>
     <row r="35" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A35" s="4" t="s">
@@ -4960,12 +4938,6 @@
       <c r="G35" s="5">
         <v>0.95831484749990903</v>
       </c>
-      <c r="K35" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="L35" s="3" t="s">
-        <v>31</v>
-      </c>
     </row>
     <row r="36" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A36" s="4" t="s">
@@ -4989,12 +4961,6 @@
       <c r="G36" s="5">
         <v>1</v>
       </c>
-      <c r="K36" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="L36" s="3" t="s">
-        <v>31</v>
-      </c>
     </row>
     <row r="37" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A37" s="4" t="s">
@@ -5018,12 +4984,6 @@
       <c r="G37" s="5">
         <v>0.32287320150037802</v>
       </c>
-      <c r="K37" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="L37" s="3" t="s">
-        <v>32</v>
-      </c>
     </row>
     <row r="38" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A38" s="4" t="s">
@@ -5047,12 +5007,6 @@
       <c r="G38" s="5">
         <v>0.92717264994552995</v>
       </c>
-      <c r="K38" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="L38" s="3" t="s">
-        <v>31</v>
-      </c>
     </row>
     <row r="39" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A39" s="4" t="s">
@@ -5076,12 +5030,6 @@
       <c r="G39" s="5">
         <v>0.87070707070706999</v>
       </c>
-      <c r="K39" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="L39" s="3" t="s">
-        <v>32</v>
-      </c>
     </row>
     <row r="40" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A40" s="4" t="s">
@@ -5105,15 +5053,6 @@
       <c r="G40" s="5">
         <v>0.50213950485175096</v>
       </c>
-      <c r="K40" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="L40" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="M40" s="3" t="s">
-        <v>33</v>
-      </c>
     </row>
     <row r="41" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A41" s="4" t="s">
@@ -5137,12 +5076,6 @@
       <c r="G41" s="5">
         <v>0.41656576663693501</v>
       </c>
-      <c r="K41" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="L41" s="3" t="s">
-        <v>31</v>
-      </c>
     </row>
     <row r="42" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A42" s="4" t="s">
@@ -5166,12 +5099,6 @@
       <c r="G42" s="5">
         <v>0.88662628383626696</v>
       </c>
-      <c r="K42" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="L42" s="3" t="s">
-        <v>32</v>
-      </c>
     </row>
     <row r="43" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A43" s="4" t="s">
@@ -5195,12 +5122,6 @@
       <c r="G43" s="5">
         <v>0.88662628383626696</v>
       </c>
-      <c r="K43" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="L43" s="3" t="s">
-        <v>32</v>
-      </c>
     </row>
     <row r="44" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A44" s="4" t="s">
@@ -5224,12 +5145,6 @@
       <c r="G44" s="5">
         <v>0.84270097160038404</v>
       </c>
-      <c r="K44" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="L44" s="3" t="s">
-        <v>32</v>
-      </c>
     </row>
     <row r="45" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A45" s="4" t="s">
@@ -5252,36 +5167,6 @@
       </c>
       <c r="G45" s="5">
         <v>0.65141719549690702</v>
-      </c>
-      <c r="K45" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="L45" s="3" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="46" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="K46" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="L46" s="3" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="47" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="K47" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="L47" s="3" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="48" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="K48" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="L48" s="3" t="s">
-        <v>31</v>
       </c>
     </row>
   </sheetData>
@@ -5290,12 +5175,12 @@
     <mergeCell ref="I1:O1"/>
     <mergeCell ref="A24:G24"/>
   </mergeCells>
-  <conditionalFormatting sqref="A1:O1048576">
-    <cfRule type="colorScale" priority="4">
+  <conditionalFormatting sqref="A1:O29 A49:O1048576 A30:J48 M30:O48">
+    <cfRule type="colorScale" priority="2">
       <colorScale>
-        <cfvo type="min"/>
+        <cfvo type="num" val="0"/>
         <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
+        <cfvo type="num" val="1"/>
         <color rgb="FFF8696B"/>
         <color rgb="FFFFEB84"/>
         <color rgb="FF63BE7B"/>
@@ -5311,11 +5196,11 @@
         <color rgb="FF63BE7B"/>
       </colorScale>
     </cfRule>
-    <cfRule type="colorScale" priority="2">
+    <cfRule type="colorScale" priority="4">
       <colorScale>
-        <cfvo type="num" val="0"/>
+        <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
-        <cfvo type="num" val="1"/>
+        <cfvo type="max"/>
         <color rgb="FFF8696B"/>
         <color rgb="FFFFEB84"/>
         <color rgb="FF63BE7B"/>
@@ -5337,4 +5222,202 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE05FBB1-52FD-4982-866C-272CD8759DE0}">
+  <dimension ref="A1:B19"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="20.85546875" customWidth="1"/>
+    <col min="2" max="2" width="14.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="A1:B19">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="num" val="1"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="num" val="100"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="3">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>